<commit_message>
Se agrego el diccionario de variables
</commit_message>
<xml_diff>
--- a/Momento 1/Prueba de escritorio.xlsx
+++ b/Momento 1/Prueba de escritorio.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10917"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10920"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/carlosguette/Documents/CESDE/Logica de programacion/Entregables/Momento 1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F1418575-320B-E64A-A1EC-418A6DBA3306}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BF953F2-7D09-8D4F-8457-85EBD24B334C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{56424B99-6AF0-E142-8D57-CDCCB118FEF6}"/>
+    <workbookView xWindow="15120" yWindow="680" windowWidth="15140" windowHeight="17780" activeTab="1" xr2:uid="{56424B99-6AF0-E142-8D57-CDCCB118FEF6}"/>
   </bookViews>
   <sheets>
-    <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
+    <sheet name="Prueba de escritorio" sheetId="1" r:id="rId1"/>
+    <sheet name="Hoja1" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="43">
   <si>
     <t>Algoritmo valor de prueba Minimo = 20, Maximo = 100, Actual = 15</t>
   </si>
@@ -138,6 +139,36 @@
   </si>
   <si>
     <t>Suggar</t>
+  </si>
+  <si>
+    <t>Nombre de la variable</t>
+  </si>
+  <si>
+    <t>Tipo de dato</t>
+  </si>
+  <si>
+    <t>Momento</t>
+  </si>
+  <si>
+    <t>Cadena</t>
+  </si>
+  <si>
+    <t>Entrada</t>
+  </si>
+  <si>
+    <t>minimumStock</t>
+  </si>
+  <si>
+    <t>Real</t>
+  </si>
+  <si>
+    <t>maximumStock</t>
+  </si>
+  <si>
+    <t>Logico</t>
+  </si>
+  <si>
+    <t>Proceso y salida</t>
   </si>
 </sst>
 </file>
@@ -218,13 +249,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -559,7 +592,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B676BC4-4BBB-7E48-85B7-7331F6FB771A}">
-  <dimension ref="A1:M25"/>
+  <dimension ref="A1:F25"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="77.83203125" bestFit="1" customWidth="1"/>
@@ -567,547 +600,578 @@
     <col min="6" max="6" width="16.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
-      <c r="K1" s="1"/>
-      <c r="L1" s="1"/>
-      <c r="M1" s="1"/>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A2" s="5" t="s">
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A2" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="G2" s="1"/>
-      <c r="H2" s="1"/>
-      <c r="I2" s="1"/>
-      <c r="J2" s="1"/>
-      <c r="K2" s="1"/>
-      <c r="L2" s="1"/>
-      <c r="M2" s="1"/>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A3" s="2" t="s">
+      <c r="B2" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="G3" s="1"/>
-      <c r="H3" s="1"/>
-      <c r="I3" s="1"/>
-      <c r="J3" s="1"/>
-      <c r="K3" s="1"/>
-      <c r="L3" s="1"/>
-      <c r="M3" s="1"/>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A4" s="2" t="s">
+      <c r="B3" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="G4" s="1"/>
-      <c r="H4" s="1"/>
-      <c r="I4" s="1"/>
-      <c r="J4" s="1"/>
-      <c r="K4" s="1"/>
-      <c r="L4" s="1"/>
-      <c r="M4" s="1"/>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A5" s="2" t="s">
+      <c r="B4" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A5" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="G5" s="1"/>
-      <c r="H5" s="1"/>
-      <c r="I5" s="1"/>
-      <c r="J5" s="1"/>
-      <c r="K5" s="1"/>
-      <c r="L5" s="1"/>
-      <c r="M5" s="1"/>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A6" s="2" t="s">
+      <c r="B5" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A6" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="G6" s="1"/>
-      <c r="H6" s="1"/>
-      <c r="I6" s="1"/>
-      <c r="J6" s="1"/>
-      <c r="K6" s="1"/>
-      <c r="L6" s="1"/>
-      <c r="M6" s="1"/>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A7" s="2" t="s">
+      <c r="B6" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A7" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="G7" s="1"/>
-      <c r="H7" s="1"/>
-      <c r="I7" s="1"/>
-      <c r="J7" s="1"/>
-      <c r="K7" s="1"/>
-      <c r="L7" s="1"/>
-      <c r="M7" s="1"/>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A8" s="2" t="s">
+      <c r="B7" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A8" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B8" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A9" s="2" t="s">
+      <c r="B8" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A9" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="F9" s="2" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A10" s="2" t="s">
+      <c r="B9" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A10" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B10" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="F10" s="2" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A11" s="2" t="s">
+      <c r="B10" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A11" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B11" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="F11" s="2" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A12" s="2" t="s">
+      <c r="B11" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A12" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B12" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="F12" s="2" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A13" s="2" t="s">
+      <c r="B12" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A13" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B13" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A14" s="2" t="s">
+      <c r="B13" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A14" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B14" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="C14" s="2">
+      <c r="B14" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C14" s="1">
         <v>20</v>
       </c>
-      <c r="D14" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="F14" s="2" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A15" s="2" t="s">
+      <c r="D14" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A15" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B15" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="C15" s="2">
+      <c r="B15" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C15" s="1">
         <v>20</v>
       </c>
-      <c r="D15" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="E15" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="F15" s="2" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A16" s="2" t="s">
+      <c r="D15" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A16" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B16" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="C16" s="2">
+      <c r="B16" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C16" s="1">
         <v>20</v>
       </c>
-      <c r="D16" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="E16" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="F16" s="2" t="s">
+      <c r="D16" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="F16" s="1" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A17" s="2" t="s">
+      <c r="A17" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B17" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="C17" s="2">
+      <c r="B17" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C17" s="1">
         <v>20</v>
       </c>
-      <c r="D17" s="2">
+      <c r="D17" s="1">
         <v>100</v>
       </c>
-      <c r="E17" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="F17" s="2" t="s">
+      <c r="E17" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="F17" s="1" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A18" s="2" t="s">
+      <c r="A18" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B18" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="C18" s="2">
+      <c r="B18" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C18" s="1">
         <v>20</v>
       </c>
-      <c r="D18" s="2">
+      <c r="D18" s="1">
         <v>100</v>
       </c>
-      <c r="E18" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="F18" s="2" t="s">
+      <c r="E18" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="F18" s="1" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A19" s="2" t="s">
+      <c r="A19" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B19" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="C19" s="2">
+      <c r="B19" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C19" s="1">
         <v>20</v>
       </c>
-      <c r="D19" s="2">
+      <c r="D19" s="1">
         <v>100</v>
       </c>
-      <c r="E19" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="F19" s="2" t="s">
+      <c r="E19" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="F19" s="1" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A20" s="2" t="s">
+      <c r="A20" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B20" s="2">
+      <c r="B20" s="1">
         <v>15</v>
       </c>
-      <c r="C20" s="2">
+      <c r="C20" s="1">
         <v>20</v>
       </c>
-      <c r="D20" s="2">
+      <c r="D20" s="1">
         <v>100</v>
       </c>
-      <c r="E20" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="F20" s="2" t="s">
+      <c r="E20" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="F20" s="1" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A21" s="2" t="s">
+      <c r="A21" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B21" s="2">
+      <c r="B21" s="1">
         <v>15</v>
       </c>
-      <c r="C21" s="2">
+      <c r="C21" s="1">
         <v>20</v>
       </c>
-      <c r="D21" s="2">
+      <c r="D21" s="1">
         <v>100</v>
       </c>
-      <c r="E21" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="F21" s="2" t="s">
+      <c r="E21" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="F21" s="1" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A22" s="2" t="s">
+      <c r="A22" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B22" s="2">
+      <c r="B22" s="1">
         <v>15</v>
       </c>
-      <c r="C22" s="2">
+      <c r="C22" s="1">
         <v>20</v>
       </c>
-      <c r="D22" s="2">
+      <c r="D22" s="1">
         <v>100</v>
       </c>
-      <c r="E22" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="F22" s="2" t="s">
+      <c r="E22" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="F22" s="1" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A23" s="2" t="s">
+      <c r="A23" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B23" s="2">
+      <c r="B23" s="1">
         <v>15</v>
       </c>
-      <c r="C23" s="2">
+      <c r="C23" s="1">
         <v>20</v>
       </c>
-      <c r="D23" s="2">
+      <c r="D23" s="1">
         <v>100</v>
       </c>
-      <c r="E23" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="F23" s="2" t="b">
+      <c r="E23" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="F23" s="1" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A24" s="2" t="s">
+      <c r="A24" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="B24" s="2">
+      <c r="B24" s="1">
         <v>15</v>
       </c>
-      <c r="C24" s="2">
+      <c r="C24" s="1">
         <v>20</v>
       </c>
-      <c r="D24" s="2">
+      <c r="D24" s="1">
         <v>100</v>
       </c>
-      <c r="E24" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="F24" s="2" t="b">
+      <c r="E24" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="F24" s="1" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A25" s="4" t="s">
+      <c r="A25" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B25" s="4"/>
-      <c r="C25" s="4"/>
-      <c r="D25" s="4"/>
-      <c r="E25" s="4"/>
-      <c r="F25" s="4"/>
+      <c r="B25" s="3"/>
+      <c r="C25" s="3"/>
+      <c r="D25" s="3"/>
+      <c r="E25" s="3"/>
+      <c r="F25" s="3"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6952BA35-1F50-9A41-9BB1-C99D07B3B204}">
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="18.83203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A1" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A2" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A3" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A4" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A5" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A6" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>42</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>